<commit_message>
Updated locations and created py file
</commit_message>
<xml_diff>
--- a/data/Regionalligen26_27.xlsx
+++ b/data/Regionalligen26_27.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alle Dokumente\Studium\Master\2. Semester\NMC - Naturinspirierte Methoden der Computerintelligenz\Datensammlung\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenna\Documents\Studium\Master\2. Semester\Natürliche Methoden der Computerintelligenz\ComputerintelligenzRegionalligen\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE4F46B-9AC8-42F5-A117-668756F2E486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F4332C-B230-4C00-8B84-4154C5420496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F32217A0-AE29-4F45-B8F3-801574AB2498}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F32217A0-AE29-4F45-B8F3-801574AB2498}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="266">
   <si>
     <t>Regio Nordost</t>
   </si>
@@ -497,9 +497,6 @@
     <t>Akon Arena</t>
   </si>
   <si>
-    <t>FC Bayern Machern II</t>
-  </si>
-  <si>
     <t>Grünwalder Stadion</t>
   </si>
   <si>
@@ -590,9 +587,6 @@
     <t>50.9601, 11.0373</t>
   </si>
   <si>
-    <t>51.4654. 11.9622</t>
-  </si>
-  <si>
     <t>50.8421, 12.9456</t>
   </si>
   <si>
@@ -837,6 +831,15 @@
   </si>
   <si>
     <t>49.2668, 11.2991 / 49.9703, 9.1301 / 49.2325, 12.6774</t>
+  </si>
+  <si>
+    <t>51,4654, 11,9622</t>
+  </si>
+  <si>
+    <t>FC Bayern München II</t>
+  </si>
+  <si>
+    <t>52,3666, 14,036</t>
   </si>
 </sst>
 </file>
@@ -917,7 +920,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -930,14 +933,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -945,14 +955,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1300,12 +1302,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -1318,9 +1320,8 @@
         <v>3</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E3" s="13"/>
+        <v>175</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -1333,9 +1334,9 @@
         <v>4</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="E4" s="14"/>
+        <v>176</v>
+      </c>
+      <c r="E4" s="6"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -1349,7 +1350,7 @@
         <v>6</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1364,9 +1365,9 @@
         <v>8</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="E6" s="14"/>
+        <v>178</v>
+      </c>
+      <c r="E6" s="6"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -1380,9 +1381,9 @@
         <v>23</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="E7" s="14"/>
+        <v>179</v>
+      </c>
+      <c r="E7" s="6"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -1396,9 +1397,9 @@
         <v>24</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="E8" s="14"/>
+        <v>263</v>
+      </c>
+      <c r="E8" s="6"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -1412,9 +1413,9 @@
         <v>25</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="E9" s="14"/>
+        <v>180</v>
+      </c>
+      <c r="E9" s="6"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -1425,12 +1426,12 @@
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="E10" s="14"/>
+        <v>265</v>
+      </c>
+      <c r="E10" s="6"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -1444,9 +1445,9 @@
         <v>26</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="E11" s="14"/>
+        <v>181</v>
+      </c>
+      <c r="E11" s="6"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -1460,9 +1461,9 @@
         <v>27</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="E12" s="14"/>
+        <v>185</v>
+      </c>
+      <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -1476,9 +1477,9 @@
         <v>28</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="E13" s="14"/>
+        <v>186</v>
+      </c>
+      <c r="E13" s="6"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -1492,9 +1493,9 @@
         <v>33</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="E14" s="14"/>
+        <v>187</v>
+      </c>
+      <c r="E14" s="6"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -1508,9 +1509,9 @@
         <v>29</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="E15" s="14"/>
+        <v>189</v>
+      </c>
+      <c r="E15" s="6"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -1521,12 +1522,12 @@
         <v>18</v>
       </c>
       <c r="C16" t="s">
+        <v>188</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="E16" s="14"/>
+      <c r="E16" s="6"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
@@ -1540,9 +1541,9 @@
         <v>30</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="E17" s="14"/>
+        <v>191</v>
+      </c>
+      <c r="E17" s="6"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
@@ -1556,9 +1557,9 @@
         <v>22</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="E18" s="14"/>
+        <v>192</v>
+      </c>
+      <c r="E18" s="6"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
@@ -1572,39 +1573,39 @@
         <v>31</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="E19" s="14"/>
+        <v>193</v>
+      </c>
+      <c r="E19" s="6"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>186</v>
-      </c>
       <c r="D20" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
+      <c r="A22" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
@@ -1617,9 +1618,8 @@
         <v>3</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E30" s="13"/>
+        <v>175</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
@@ -1632,9 +1632,9 @@
         <v>36</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="E31" s="14"/>
+        <v>196</v>
+      </c>
+      <c r="E31" s="6"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
@@ -1648,9 +1648,9 @@
         <v>37</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="E32" s="14"/>
+        <v>195</v>
+      </c>
+      <c r="E32" s="6"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
@@ -1664,9 +1664,9 @@
         <v>39</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="E33" s="14"/>
+        <v>209</v>
+      </c>
+      <c r="E33" s="6"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
@@ -1680,9 +1680,9 @@
         <v>41</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="E34" s="14"/>
+        <v>210</v>
+      </c>
+      <c r="E34" s="6"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
@@ -1696,9 +1696,9 @@
         <v>43</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="E35" s="14"/>
+        <v>211</v>
+      </c>
+      <c r="E35" s="6"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
@@ -1712,9 +1712,9 @@
         <v>74</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="E36" s="14"/>
+        <v>197</v>
+      </c>
+      <c r="E36" s="6"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
@@ -1728,9 +1728,9 @@
         <v>46</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="E37" s="14"/>
+        <v>198</v>
+      </c>
+      <c r="E37" s="6"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
@@ -1744,9 +1744,9 @@
         <v>48</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E38" s="14"/>
+        <v>199</v>
+      </c>
+      <c r="E38" s="6"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
@@ -1760,9 +1760,9 @@
         <v>50</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="E39" s="14"/>
+        <v>200</v>
+      </c>
+      <c r="E39" s="6"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
@@ -1776,9 +1776,9 @@
         <v>72</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="E40" s="14"/>
+        <v>201</v>
+      </c>
+      <c r="E40" s="6"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
@@ -1792,9 +1792,9 @@
         <v>53</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="E41" s="14"/>
+        <v>202</v>
+      </c>
+      <c r="E41" s="6"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
@@ -1808,9 +1808,9 @@
         <v>73</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="E42" s="14"/>
+        <v>203</v>
+      </c>
+      <c r="E42" s="6"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
@@ -1824,9 +1824,9 @@
         <v>56</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="E43" s="14"/>
+        <v>204</v>
+      </c>
+      <c r="E43" s="6"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
@@ -1840,9 +1840,9 @@
         <v>58</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="E44" s="14"/>
+        <v>205</v>
+      </c>
+      <c r="E44" s="6"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
@@ -1856,7 +1856,7 @@
         <v>63</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1871,7 +1871,7 @@
         <v>64</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -1885,7 +1885,7 @@
         <v>65</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -1899,24 +1899,24 @@
         <v>66</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="7" t="s">
+      <c r="A50" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="8" t="s">
+      <c r="A52" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="8"/>
+      <c r="B52" s="10"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
@@ -1929,9 +1929,8 @@
         <v>3</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E54" s="13"/>
+        <v>175</v>
+      </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
@@ -1944,9 +1943,9 @@
         <v>70</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="E55" s="14"/>
+        <v>212</v>
+      </c>
+      <c r="E55" s="6"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
@@ -1960,9 +1959,9 @@
         <v>76</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="E56" s="14"/>
+        <v>213</v>
+      </c>
+      <c r="E56" s="6"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
@@ -1976,9 +1975,9 @@
         <v>77</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="E57" s="14"/>
+        <v>214</v>
+      </c>
+      <c r="E57" s="6"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
@@ -1992,9 +1991,9 @@
         <v>78</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="E58" s="14"/>
+        <v>215</v>
+      </c>
+      <c r="E58" s="6"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
@@ -2008,9 +2007,9 @@
         <v>81</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="E59" s="14"/>
+        <v>216</v>
+      </c>
+      <c r="E59" s="6"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
@@ -2024,9 +2023,9 @@
         <v>83</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="E60" s="14"/>
+        <v>217</v>
+      </c>
+      <c r="E60" s="6"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
@@ -2040,9 +2039,9 @@
         <v>85</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="E61" s="14"/>
+        <v>218</v>
+      </c>
+      <c r="E61" s="6"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
@@ -2056,9 +2055,9 @@
         <v>87</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="E62" s="14"/>
+        <v>219</v>
+      </c>
+      <c r="E62" s="6"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
@@ -2072,9 +2071,9 @@
         <v>89</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="E63" s="14"/>
+        <v>220</v>
+      </c>
+      <c r="E63" s="6"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
@@ -2088,9 +2087,9 @@
         <v>91</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="E64" s="14"/>
+        <v>221</v>
+      </c>
+      <c r="E64" s="6"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
@@ -2104,9 +2103,9 @@
         <v>93</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="E65" s="14"/>
+        <v>222</v>
+      </c>
+      <c r="E65" s="6"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
@@ -2120,9 +2119,9 @@
         <v>95</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="E66" s="14"/>
+        <v>223</v>
+      </c>
+      <c r="E66" s="6"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
@@ -2136,7 +2135,7 @@
         <v>97</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
@@ -2151,7 +2150,7 @@
         <v>100</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -2166,7 +2165,7 @@
         <v>103</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
@@ -2181,24 +2180,24 @@
         <v>104</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="7" t="s">
+      <c r="A72" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B72" s="7"/>
-      <c r="C72" s="7"/>
-      <c r="D72" s="7"/>
+      <c r="B72" s="8"/>
+      <c r="C72" s="8"/>
+      <c r="D72" s="8"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="9" t="s">
+      <c r="A78" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="B78" s="9"/>
-      <c r="C78" s="9"/>
-      <c r="D78" s="9"/>
+      <c r="B78" s="12"/>
+      <c r="C78" s="12"/>
+      <c r="D78" s="12"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
@@ -2211,9 +2210,8 @@
         <v>3</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E80" s="13"/>
+        <v>175</v>
+      </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81">
@@ -2226,9 +2224,9 @@
         <v>108</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E81" s="14"/>
+        <v>228</v>
+      </c>
+      <c r="E81" s="6"/>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82">
@@ -2242,9 +2240,9 @@
         <v>110</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="E82" s="14"/>
+        <v>229</v>
+      </c>
+      <c r="E82" s="6"/>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83">
@@ -2258,9 +2256,9 @@
         <v>112</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="E83" s="14"/>
+        <v>230</v>
+      </c>
+      <c r="E83" s="6"/>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84">
@@ -2274,9 +2272,9 @@
         <v>114</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="E84" s="14"/>
+        <v>231</v>
+      </c>
+      <c r="E84" s="6"/>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85">
@@ -2290,9 +2288,9 @@
         <v>116</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="E85" s="14"/>
+        <v>232</v>
+      </c>
+      <c r="E85" s="6"/>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86">
@@ -2306,9 +2304,9 @@
         <v>118</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="E86" s="14"/>
+        <v>233</v>
+      </c>
+      <c r="E86" s="6"/>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87">
@@ -2322,9 +2320,9 @@
         <v>120</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="E87" s="14"/>
+        <v>234</v>
+      </c>
+      <c r="E87" s="6"/>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88">
@@ -2338,9 +2336,9 @@
         <v>122</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="E88" s="14"/>
+        <v>235</v>
+      </c>
+      <c r="E88" s="6"/>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89">
@@ -2354,9 +2352,9 @@
         <v>138</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="E89" s="14"/>
+        <v>236</v>
+      </c>
+      <c r="E89" s="6"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90">
@@ -2370,9 +2368,9 @@
         <v>125</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="E90" s="14"/>
+        <v>237</v>
+      </c>
+      <c r="E90" s="6"/>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91">
@@ -2386,9 +2384,9 @@
         <v>137</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="E91" s="14"/>
+        <v>238</v>
+      </c>
+      <c r="E91" s="6"/>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92">
@@ -2402,9 +2400,9 @@
         <v>128</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="E92" s="14"/>
+        <v>239</v>
+      </c>
+      <c r="E92" s="6"/>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
@@ -2418,7 +2416,7 @@
         <v>130</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
@@ -2433,7 +2431,7 @@
         <v>136</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
@@ -2448,7 +2446,7 @@
         <v>133</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
@@ -2463,25 +2461,25 @@
         <v>135</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="I96" s="5"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="6" t="s">
+      <c r="A98" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="B98" s="6"/>
-      <c r="C98" s="6"/>
-      <c r="D98" s="6"/>
+      <c r="B98" s="11"/>
+      <c r="C98" s="11"/>
+      <c r="D98" s="11"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="10" t="s">
+      <c r="A100" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="B100" s="10"/>
-      <c r="C100" s="10"/>
-      <c r="D100" s="10"/>
+      <c r="B100" s="13"/>
+      <c r="C100" s="13"/>
+      <c r="D100" s="13"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
@@ -2494,9 +2492,8 @@
         <v>3</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E102" s="13"/>
+        <v>175</v>
+      </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
@@ -2509,7 +2506,7 @@
         <v>150</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
@@ -2524,9 +2521,9 @@
         <v>142</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="E104" s="14"/>
+        <v>243</v>
+      </c>
+      <c r="E104" s="6"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105">
@@ -2537,12 +2534,12 @@
         <v>143</v>
       </c>
       <c r="C105" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="E105" s="14"/>
+        <v>244</v>
+      </c>
+      <c r="E105" s="6"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106">
@@ -2556,9 +2553,9 @@
         <v>145</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="E106" s="14"/>
+        <v>245</v>
+      </c>
+      <c r="E106" s="6"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107">
@@ -2572,9 +2569,9 @@
         <v>147</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="E107" s="14"/>
+        <v>246</v>
+      </c>
+      <c r="E107" s="6"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108">
@@ -2585,12 +2582,12 @@
         <v>148</v>
       </c>
       <c r="C108" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="E108" s="14"/>
+        <v>247</v>
+      </c>
+      <c r="E108" s="6"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109">
@@ -2598,15 +2595,15 @@
         <v>7</v>
       </c>
       <c r="B109" t="s">
+        <v>154</v>
+      </c>
+      <c r="C109" t="s">
         <v>155</v>
       </c>
-      <c r="C109" t="s">
-        <v>156</v>
-      </c>
       <c r="D109" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="E109" s="14"/>
+        <v>248</v>
+      </c>
+      <c r="E109" s="6"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110">
@@ -2614,15 +2611,15 @@
         <v>8</v>
       </c>
       <c r="B110" t="s">
+        <v>156</v>
+      </c>
+      <c r="C110" t="s">
         <v>157</v>
       </c>
-      <c r="C110" t="s">
-        <v>158</v>
-      </c>
       <c r="D110" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="E110" s="14"/>
+        <v>249</v>
+      </c>
+      <c r="E110" s="6"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111">
@@ -2630,15 +2627,15 @@
         <v>9</v>
       </c>
       <c r="B111" t="s">
+        <v>264</v>
+      </c>
+      <c r="C111" t="s">
         <v>151</v>
       </c>
-      <c r="C111" t="s">
-        <v>152</v>
-      </c>
       <c r="D111" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E111" s="14"/>
+        <v>250</v>
+      </c>
+      <c r="E111" s="6"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112">
@@ -2646,15 +2643,15 @@
         <v>10</v>
       </c>
       <c r="B112" t="s">
+        <v>158</v>
+      </c>
+      <c r="C112" t="s">
         <v>159</v>
       </c>
-      <c r="C112" t="s">
-        <v>160</v>
-      </c>
       <c r="D112" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="E112" s="14"/>
+        <v>251</v>
+      </c>
+      <c r="E112" s="6"/>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113">
@@ -2662,15 +2659,15 @@
         <v>11</v>
       </c>
       <c r="B113" t="s">
+        <v>160</v>
+      </c>
+      <c r="C113" t="s">
         <v>161</v>
       </c>
-      <c r="C113" t="s">
-        <v>162</v>
-      </c>
       <c r="D113" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="E113" s="14"/>
+        <v>252</v>
+      </c>
+      <c r="E113" s="6"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114">
@@ -2678,15 +2675,15 @@
         <v>12</v>
       </c>
       <c r="B114" t="s">
+        <v>162</v>
+      </c>
+      <c r="C114" t="s">
         <v>163</v>
       </c>
-      <c r="C114" t="s">
-        <v>164</v>
-      </c>
       <c r="D114" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="E114" s="14"/>
+        <v>253</v>
+      </c>
+      <c r="E114" s="6"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
@@ -2694,13 +2691,13 @@
         <v>13</v>
       </c>
       <c r="B115" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="C115" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="C115" s="1" t="s">
-        <v>174</v>
-      </c>
       <c r="D115" s="4" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
@@ -2709,15 +2706,15 @@
         <v>14</v>
       </c>
       <c r="B116" t="s">
+        <v>166</v>
+      </c>
+      <c r="C116" t="s">
         <v>167</v>
       </c>
-      <c r="C116" t="s">
-        <v>168</v>
-      </c>
       <c r="D116" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="E116" s="14"/>
+        <v>254</v>
+      </c>
+      <c r="E116" s="6"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117">
@@ -2725,15 +2722,15 @@
         <v>15</v>
       </c>
       <c r="B117" t="s">
+        <v>168</v>
+      </c>
+      <c r="C117" t="s">
         <v>169</v>
       </c>
-      <c r="C117" t="s">
-        <v>170</v>
-      </c>
       <c r="D117" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="E117" s="14"/>
+        <v>255</v>
+      </c>
+      <c r="E117" s="6"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118">
@@ -2741,50 +2738,50 @@
         <v>16</v>
       </c>
       <c r="B118" t="s">
+        <v>170</v>
+      </c>
+      <c r="C118" t="s">
         <v>171</v>
       </c>
-      <c r="C118" t="s">
-        <v>172</v>
-      </c>
       <c r="D118" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="E118" s="14"/>
+        <v>256</v>
+      </c>
+      <c r="E118" s="6"/>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>17</v>
       </c>
       <c r="B119" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C119" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="C119" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="D119" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="B121" s="7"/>
-      <c r="C121" s="7"/>
-      <c r="D121" s="7"/>
+      <c r="A121" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B121" s="8"/>
+      <c r="C121" s="8"/>
+      <c r="D121" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A98:D98"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="A100:D100"/>
+    <mergeCell ref="A121:D121"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="A50:D50"/>
     <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A98:D98"/>
-    <mergeCell ref="A78:D78"/>
-    <mergeCell ref="A100:D100"/>
-    <mergeCell ref="A121:D121"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="55" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
corrected coords and clubs and renewed Strategy and Population algorithm
</commit_message>
<xml_diff>
--- a/data/Regionalligen26_27.xlsx
+++ b/data/Regionalligen26_27.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenna\Documents\Studium\Master\2. Semester\Natürliche Methoden der Computerintelligenz\ComputerintelligenzRegionalligen\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alle Dokumente\Studium\Master\2. Semester\NMC - Naturinspirierte Methoden der Computerintelligenz\Python-Implementierungen\Projekt_kompassmodell\ComputerintelligenzRegionalligen\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F4332C-B230-4C00-8B84-4154C5420496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C633A8E-56E7-4DF2-A765-C7CAD9074D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F32217A0-AE29-4F45-B8F3-801574AB2498}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F32217A0-AE29-4F45-B8F3-801574AB2498}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="250">
   <si>
     <t>Regio Nordost</t>
   </si>
@@ -221,24 +221,12 @@
     <t>Städtisches Stadion an der Düsternortstraße</t>
   </si>
   <si>
-    <t>1. FC Germania Egestorf/Langreder</t>
-  </si>
-  <si>
-    <t>Blumenthaler SV</t>
-  </si>
-  <si>
     <t>Eimsbütteler TV</t>
   </si>
   <si>
     <t>SV Todesfelde</t>
   </si>
   <si>
-    <t>Stadion an der Ammerke</t>
-  </si>
-  <si>
-    <t>Burgwall-Stadion</t>
-  </si>
-  <si>
     <t>ETV-Sportzentrum Hoheluft</t>
   </si>
   <si>
@@ -332,21 +320,6 @@
     <t>Mondpalast-Arena</t>
   </si>
   <si>
-    <t>SV Bergisch Gladbach / Siegburger SV</t>
-  </si>
-  <si>
-    <t>BELKAW-Arena / Walter-Mundorf-Stadion</t>
-  </si>
-  <si>
-    <t>VfB 03 Hilden / Ratingen 04/19</t>
-  </si>
-  <si>
-    <t>abhängig von Aufstiegsspielen (07.06.)</t>
-  </si>
-  <si>
-    <t>Sportanlage Hoffeldstraße / Stadion Ratingen</t>
-  </si>
-  <si>
     <t>Westfalia Rhynern</t>
   </si>
   <si>
@@ -359,9 +332,6 @@
     <t>Lohrheidestadion</t>
   </si>
   <si>
-    <t>Liga-Ende am 07.06.</t>
-  </si>
-  <si>
     <t>Regio Südwest</t>
   </si>
   <si>
@@ -440,18 +410,6 @@
     <t>Eintracht Frankfurt II</t>
   </si>
   <si>
-    <t>1. FC Kaiserslautern II / FK Pirmasens</t>
-  </si>
-  <si>
-    <t>Fritz-Walter-Stadion Platz 4 / Sportpark Husterhöhe</t>
-  </si>
-  <si>
-    <t>VfR Mannheim / FC Eddersheim / FK Pirmasens / 1. FC Kaiserslautern II</t>
-  </si>
-  <si>
-    <t>Rhein-Neckar-Stadion / Sportplatz Mönchhofstraße / Sportpark Husterhöhe / Fritz-Walter-Stadion Platz 4</t>
-  </si>
-  <si>
     <t>Maxworx-Sportpark</t>
   </si>
   <si>
@@ -491,12 +449,6 @@
     <t>DJK Vilzing</t>
   </si>
   <si>
-    <t>Würzburger Kickers</t>
-  </si>
-  <si>
-    <t>Akon Arena</t>
-  </si>
-  <si>
     <t>Grünwalder Stadion</t>
   </si>
   <si>
@@ -536,12 +488,6 @@
     <t>SMR-Arena</t>
   </si>
   <si>
-    <t>FC Memmingen</t>
-  </si>
-  <si>
-    <t>Memminger Arena</t>
-  </si>
-  <si>
     <t>TSV Schwaben Augsburg</t>
   </si>
   <si>
@@ -560,12 +506,6 @@
     <t>3C Sportpark Landsberg</t>
   </si>
   <si>
-    <t>SpVgg Greuther Fürth II / Viktoria Aschaffenburg / ASV Cham</t>
-  </si>
-  <si>
-    <t>M. A. R Arena / Stadion am Schönbusch / Kappenberger Sportzentrum im Quader</t>
-  </si>
-  <si>
     <t>Spree-Arena</t>
   </si>
   <si>
@@ -590,15 +530,6 @@
     <t>50.8421, 12.9456</t>
   </si>
   <si>
-    <t>Hertha BSC II</t>
-  </si>
-  <si>
-    <t>abhängig von Aufstiegsspiel - falls Aufstieg, rutscht Hertha II von unten wieder rein (01.06.)</t>
-  </si>
-  <si>
-    <t>Stadion auf dem Wurfplatz</t>
-  </si>
-  <si>
     <t>52.4327, 13.3547</t>
   </si>
   <si>
@@ -626,9 +557,6 @@
     <t>52.3900, 13.1924</t>
   </si>
   <si>
-    <t>52.5172, 13.2367</t>
-  </si>
-  <si>
     <t>53.7038, 9.3805</t>
   </si>
   <si>
@@ -662,12 +590,6 @@
     <t>53.0385, 8.6431</t>
   </si>
   <si>
-    <t>52.2860, 9.5122</t>
-  </si>
-  <si>
-    <t>53.1880, 8.5836</t>
-  </si>
-  <si>
     <t>53.5892, 9.9686</t>
   </si>
   <si>
@@ -722,12 +644,6 @@
     <t>51.4858, 7.1186</t>
   </si>
   <si>
-    <t>51,1736, 6.9345 / 51.2955, 6.8404</t>
-  </si>
-  <si>
-    <t>50.9937, 7.1200 / 50.8059, 7.2186</t>
-  </si>
-  <si>
     <t>48.4045, 10.0095</t>
   </si>
   <si>
@@ -818,21 +734,9 @@
     <t>53.8976,  10.1853</t>
   </si>
   <si>
-    <t>47.9792, 10.1651</t>
-  </si>
-  <si>
     <t>49.4346, 7.7801 / 49.2185, 7.6075</t>
   </si>
   <si>
-    <t>49.4787, 8.5005 / 50.0422, 8.4762 / 49.2185, 7.6075 / 49.4346, 7.7801</t>
-  </si>
-  <si>
-    <t>abhängig von Aufstiegsspiel - falls Aufstieg, rutscht Memmingen von unten wieder rein (01.06.); Relegationsspiele bis zum 01.06.</t>
-  </si>
-  <si>
-    <t>49.2668, 11.2991 / 49.9703, 9.1301 / 49.2325, 12.6774</t>
-  </si>
-  <si>
     <t>51,4654, 11,9622</t>
   </si>
   <si>
@@ -840,6 +744,54 @@
   </si>
   <si>
     <t>52,3666, 14,036</t>
+  </si>
+  <si>
+    <t>SV Bergisch Gladbach</t>
+  </si>
+  <si>
+    <t>VfB 03 Hilden</t>
+  </si>
+  <si>
+    <t>BELKAW-Arena</t>
+  </si>
+  <si>
+    <t>Sportanlage Hoffeldstraße</t>
+  </si>
+  <si>
+    <t>50.9937, 7.1200</t>
+  </si>
+  <si>
+    <t>51,1736, 6.9345</t>
+  </si>
+  <si>
+    <t>1. FC Kaiserslautern II</t>
+  </si>
+  <si>
+    <t>Fritz-Walter-Stadion Platz 4</t>
+  </si>
+  <si>
+    <t>VfR Mannheim</t>
+  </si>
+  <si>
+    <t>Rhein-Neckar-Stadion</t>
+  </si>
+  <si>
+    <t>49.4787, 8.5005</t>
+  </si>
+  <si>
+    <t>TSV 1860 München</t>
+  </si>
+  <si>
+    <t>Grünwälder Stadion</t>
+  </si>
+  <si>
+    <t>SpVgg Greuther Fürth II</t>
+  </si>
+  <si>
+    <t>M. A. R Arena</t>
+  </si>
+  <si>
+    <t>49.2668, 11.2991</t>
   </si>
 </sst>
 </file>
@@ -920,24 +872,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -946,13 +900,8 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1289,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C010D262-1EBF-4A94-BDC5-BBB2BE47A472}">
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I118"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
@@ -1302,25 +1251,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>175</v>
+      <c r="D3" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1333,24 +1282,24 @@
       <c r="C4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="E4" s="6"/>
+      <c r="D4" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="4"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="A5" s="11">
         <f>A4+1</f>
         <v>2</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>177</v>
+      <c r="D5" s="12" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1364,10 +1313,10 @@
       <c r="C6" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="E6" s="6"/>
+      <c r="D6" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" s="4"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -1380,10 +1329,10 @@
       <c r="C7" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="E7" s="6"/>
+      <c r="D7" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E7" s="4"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -1396,10 +1345,10 @@
       <c r="C8" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="E8" s="6"/>
+      <c r="D8" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E8" s="4"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -1412,10 +1361,10 @@
       <c r="C9" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="E9" s="6"/>
+      <c r="D9" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -1426,12 +1375,12 @@
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>174</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="E10" s="6"/>
+        <v>154</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -1444,10 +1393,10 @@
       <c r="C11" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="E11" s="6"/>
+      <c r="D11" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -1460,10 +1409,10 @@
       <c r="C12" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="E12" s="6"/>
+      <c r="D12" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -1476,10 +1425,10 @@
       <c r="C13" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="E13" s="6"/>
+      <c r="D13" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E13" s="4"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -1492,10 +1441,10 @@
       <c r="C14" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="E14" s="6"/>
+      <c r="D14" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="E14" s="4"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -1508,10 +1457,10 @@
       <c r="C15" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="E15" s="6"/>
+      <c r="D15" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E15" s="4"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -1522,12 +1471,12 @@
         <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>188</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="E16" s="6"/>
+        <v>165</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E16" s="4"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
@@ -1540,10 +1489,10 @@
       <c r="C17" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="E17" s="6"/>
+      <c r="D17" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E17" s="4"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
@@ -1556,10 +1505,10 @@
       <c r="C18" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="E18" s="6"/>
+      <c r="D18" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E18" s="4"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
@@ -1572,32 +1521,10 @@
       <c r="C19" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="E19" s="6"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>17</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
+      <c r="D19" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E19" s="4"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
@@ -1612,13 +1539,13 @@
         <v>1</v>
       </c>
       <c r="B30" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C30" t="s">
         <v>3</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>175</v>
+      <c r="D30" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1631,10 +1558,10 @@
       <c r="C31" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E31" s="6"/>
+      <c r="D31" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E31" s="4"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32">
@@ -1647,10 +1574,10 @@
       <c r="C32" t="s">
         <v>37</v>
       </c>
-      <c r="D32" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="E32" s="6"/>
+      <c r="D32" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E32" s="4"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33">
@@ -1663,10 +1590,10 @@
       <c r="C33" t="s">
         <v>39</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="E33" s="6"/>
+      <c r="D33" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="E33" s="4"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34">
@@ -1679,10 +1606,10 @@
       <c r="C34" t="s">
         <v>41</v>
       </c>
-      <c r="D34" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="E34" s="6"/>
+      <c r="D34" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E34" s="4"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35">
@@ -1695,10 +1622,10 @@
       <c r="C35" t="s">
         <v>43</v>
       </c>
-      <c r="D35" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="E35" s="6"/>
+      <c r="D35" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E35" s="4"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36">
@@ -1709,12 +1636,12 @@
         <v>44</v>
       </c>
       <c r="C36" t="s">
-        <v>74</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="E36" s="6"/>
+        <v>70</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E36" s="4"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37">
@@ -1727,10 +1654,10 @@
       <c r="C37" t="s">
         <v>46</v>
       </c>
-      <c r="D37" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="E37" s="6"/>
+      <c r="D37" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38">
@@ -1743,10 +1670,10 @@
       <c r="C38" t="s">
         <v>48</v>
       </c>
-      <c r="D38" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="E38" s="6"/>
+      <c r="D38" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39">
@@ -1759,10 +1686,10 @@
       <c r="C39" t="s">
         <v>50</v>
       </c>
-      <c r="D39" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="E39" s="6"/>
+      <c r="D39" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40">
@@ -1773,12 +1700,12 @@
         <v>51</v>
       </c>
       <c r="C40" t="s">
-        <v>72</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="E40" s="6"/>
+        <v>68</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E40" s="4"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41">
@@ -1791,10 +1718,10 @@
       <c r="C41" t="s">
         <v>53</v>
       </c>
-      <c r="D41" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="E41" s="6"/>
+      <c r="D41" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E41" s="4"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42">
@@ -1805,12 +1732,12 @@
         <v>54</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="E42" s="6"/>
+        <v>69</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E42" s="4"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43">
@@ -1823,10 +1750,10 @@
       <c r="C43" t="s">
         <v>56</v>
       </c>
-      <c r="D43" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="E43" s="6"/>
+      <c r="D43" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E43" s="4"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44">
@@ -1839,80 +1766,44 @@
       <c r="C44" t="s">
         <v>58</v>
       </c>
-      <c r="D44" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="E44" s="6"/>
+      <c r="D44" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="E44" s="4"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="1">
+      <c r="A45">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C45" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>206</v>
+      <c r="C45" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="1">
+      <c r="A46">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C46" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="1">
-        <v>17</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="1">
-        <v>18</v>
-      </c>
-      <c r="B48" s="1" t="s">
+      <c r="C46" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C48" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="B50" s="8"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
+      <c r="D46" s="12" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B52" s="10"/>
       <c r="C52" s="10"/>
@@ -1923,13 +1814,13 @@
         <v>1</v>
       </c>
       <c r="B54" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C54" t="s">
         <v>3</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>175</v>
+      <c r="D54" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -1937,15 +1828,15 @@
         <v>1</v>
       </c>
       <c r="B55" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C55" t="s">
-        <v>70</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="E55" s="6"/>
+        <v>66</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E55" s="4"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
@@ -1953,15 +1844,15 @@
         <v>2</v>
       </c>
       <c r="B56" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C56" t="s">
-        <v>76</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="E56" s="6"/>
+        <v>72</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="E56" s="4"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
@@ -1969,15 +1860,15 @@
         <v>3</v>
       </c>
       <c r="B57" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C57" t="s">
-        <v>77</v>
-      </c>
-      <c r="D57" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="E57" s="6"/>
+        <v>73</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E57" s="4"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
@@ -1985,15 +1876,15 @@
         <v>4</v>
       </c>
       <c r="B58" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C58" t="s">
-        <v>78</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="E58" s="6"/>
+        <v>74</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E58" s="4"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
@@ -2001,15 +1892,15 @@
         <v>5</v>
       </c>
       <c r="B59" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C59" t="s">
-        <v>81</v>
-      </c>
-      <c r="D59" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="E59" s="6"/>
+        <v>77</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E59" s="4"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
@@ -2017,15 +1908,15 @@
         <v>6</v>
       </c>
       <c r="B60" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C60" t="s">
-        <v>83</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="E60" s="6"/>
+        <v>79</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E60" s="4"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
@@ -2033,15 +1924,15 @@
         <v>7</v>
       </c>
       <c r="B61" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C61" t="s">
-        <v>85</v>
-      </c>
-      <c r="D61" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="E61" s="6"/>
+        <v>81</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="E61" s="4"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
@@ -2049,15 +1940,15 @@
         <v>8</v>
       </c>
       <c r="B62" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C62" t="s">
-        <v>87</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="E62" s="6"/>
+        <v>83</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="E62" s="4"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
@@ -2065,15 +1956,15 @@
         <v>9</v>
       </c>
       <c r="B63" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C63" t="s">
-        <v>89</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="E63" s="6"/>
+        <v>85</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E63" s="4"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
@@ -2081,15 +1972,15 @@
         <v>10</v>
       </c>
       <c r="B64" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C64" t="s">
-        <v>91</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="E64" s="6"/>
+        <v>87</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="E64" s="4"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65">
@@ -2097,15 +1988,15 @@
         <v>11</v>
       </c>
       <c r="B65" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C65" t="s">
-        <v>93</v>
-      </c>
-      <c r="D65" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="E65" s="6"/>
+        <v>89</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E65" s="4"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66">
@@ -2113,104 +2004,96 @@
         <v>12</v>
       </c>
       <c r="B66" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C66" t="s">
-        <v>95</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="E66" s="6"/>
+        <v>91</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E66" s="4"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="1">
+      <c r="A67" s="11">
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="B67" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D67" s="4" t="s">
-        <v>227</v>
+      <c r="B67" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="C67" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="1">
+      <c r="A68" s="11">
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="B68" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>226</v>
+      <c r="B68" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="C68" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="1">
+      <c r="A69" s="11">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="B69" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>224</v>
+      <c r="B69" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C69" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="1">
+      <c r="A70" s="11">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="B72" s="8"/>
-      <c r="C72" s="8"/>
-      <c r="D72" s="8"/>
+      <c r="B70" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C70" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D70" s="12" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="B78" s="12"/>
-      <c r="C78" s="12"/>
-      <c r="D78" s="12"/>
+      <c r="A78" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B78" s="6"/>
+      <c r="C78" s="6"/>
+      <c r="D78" s="6"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>1</v>
       </c>
       <c r="B80" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C80" t="s">
         <v>3</v>
       </c>
-      <c r="D80" s="2" t="s">
-        <v>175</v>
+      <c r="D80" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
@@ -2218,15 +2101,15 @@
         <v>1</v>
       </c>
       <c r="B81" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="C81" t="s">
-        <v>108</v>
-      </c>
-      <c r="D81" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="E81" s="6"/>
+        <v>98</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E81" s="4"/>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82">
@@ -2234,15 +2117,15 @@
         <v>2</v>
       </c>
       <c r="B82" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="C82" t="s">
-        <v>110</v>
-      </c>
-      <c r="D82" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="E82" s="6"/>
+        <v>100</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E82" s="4"/>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83">
@@ -2250,15 +2133,15 @@
         <v>3</v>
       </c>
       <c r="B83" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="C83" t="s">
-        <v>112</v>
-      </c>
-      <c r="D83" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E83" s="6"/>
+        <v>102</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E83" s="4"/>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84">
@@ -2266,15 +2149,15 @@
         <v>4</v>
       </c>
       <c r="B84" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="C84" t="s">
-        <v>114</v>
-      </c>
-      <c r="D84" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="E84" s="6"/>
+        <v>104</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E84" s="4"/>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85">
@@ -2282,15 +2165,15 @@
         <v>5</v>
       </c>
       <c r="B85" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C85" t="s">
-        <v>116</v>
-      </c>
-      <c r="D85" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="E85" s="6"/>
+        <v>106</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E85" s="4"/>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86">
@@ -2298,15 +2181,15 @@
         <v>6</v>
       </c>
       <c r="B86" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C86" t="s">
-        <v>118</v>
-      </c>
-      <c r="D86" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="E86" s="6"/>
+        <v>108</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="E86" s="4"/>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87">
@@ -2314,15 +2197,15 @@
         <v>7</v>
       </c>
       <c r="B87" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C87" t="s">
-        <v>120</v>
-      </c>
-      <c r="D87" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="E87" s="6"/>
+        <v>110</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E87" s="4"/>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88">
@@ -2330,15 +2213,15 @@
         <v>8</v>
       </c>
       <c r="B88" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="C88" t="s">
-        <v>122</v>
-      </c>
-      <c r="D88" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="E88" s="6"/>
+        <v>112</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="E88" s="4"/>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89">
@@ -2346,15 +2229,15 @@
         <v>9</v>
       </c>
       <c r="B89" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C89" t="s">
-        <v>138</v>
-      </c>
-      <c r="D89" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="E89" s="6"/>
+        <v>124</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E89" s="4"/>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90">
@@ -2362,15 +2245,15 @@
         <v>10</v>
       </c>
       <c r="B90" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C90" t="s">
-        <v>125</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="E90" s="6"/>
+        <v>115</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E90" s="4"/>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91">
@@ -2378,15 +2261,15 @@
         <v>11</v>
       </c>
       <c r="B91" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="C91" t="s">
-        <v>137</v>
-      </c>
-      <c r="D91" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="E91" s="6"/>
+        <v>123</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E91" s="4"/>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92">
@@ -2394,119 +2277,119 @@
         <v>12</v>
       </c>
       <c r="B92" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C92" t="s">
-        <v>128</v>
-      </c>
-      <c r="D92" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="E92" s="6"/>
+        <v>118</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E92" s="4"/>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A93" s="1">
+      <c r="A93" s="11">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
-      <c r="B93" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D93" s="4" t="s">
-        <v>240</v>
+      <c r="B93" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C93" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D93" s="12" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A94" s="1">
+      <c r="A94" s="11">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
-      <c r="B94" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="D94" s="4" t="s">
-        <v>241</v>
+      <c r="B94" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C94" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="D94" s="12" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A95" s="1">
+      <c r="A95" s="11">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
-      <c r="B95" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="D95" s="4" t="s">
-        <v>259</v>
+      <c r="B95" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="C95" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="D95" s="12" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A96" s="1">
+      <c r="A96" s="11">
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
-      <c r="B96" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="D96" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="I96" s="5"/>
+      <c r="B96" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="C96" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="D96" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="I96" s="3"/>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="B98" s="11"/>
-      <c r="C98" s="11"/>
-      <c r="D98" s="11"/>
+      <c r="A98" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B98" s="5"/>
+      <c r="C98" s="5"/>
+      <c r="D98" s="5"/>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="B100" s="13"/>
-      <c r="C100" s="13"/>
-      <c r="D100" s="13"/>
+      <c r="A100" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B100" s="7"/>
+      <c r="C100" s="7"/>
+      <c r="D100" s="7"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>1</v>
       </c>
       <c r="B102" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C102" t="s">
         <v>3</v>
       </c>
-      <c r="D102" s="2" t="s">
-        <v>175</v>
+      <c r="D102" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="1">
+      <c r="A103" s="11">
         <v>1</v>
       </c>
-      <c r="B103" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="C103" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="D103" s="4" t="s">
-        <v>242</v>
+      <c r="B103" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="C103" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="D103" s="12" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
@@ -2515,15 +2398,15 @@
         <v>2</v>
       </c>
       <c r="B104" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="C104" t="s">
-        <v>142</v>
-      </c>
-      <c r="D104" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="E104" s="6"/>
+        <v>128</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E104" s="4"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105">
@@ -2531,15 +2414,15 @@
         <v>3</v>
       </c>
       <c r="B105" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="C105" t="s">
-        <v>153</v>
-      </c>
-      <c r="D105" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="E105" s="6"/>
+        <v>137</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E105" s="4"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106">
@@ -2547,15 +2430,15 @@
         <v>4</v>
       </c>
       <c r="B106" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="C106" t="s">
-        <v>145</v>
-      </c>
-      <c r="D106" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="E106" s="6"/>
+        <v>131</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="E106" s="4"/>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107">
@@ -2563,15 +2446,15 @@
         <v>5</v>
       </c>
       <c r="B107" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="C107" t="s">
-        <v>147</v>
-      </c>
-      <c r="D107" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="E107" s="6"/>
+        <v>133</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="E107" s="4"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108">
@@ -2579,15 +2462,15 @@
         <v>6</v>
       </c>
       <c r="B108" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="C108" t="s">
-        <v>152</v>
-      </c>
-      <c r="D108" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="E108" s="6"/>
+        <v>136</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="E108" s="4"/>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109">
@@ -2595,15 +2478,15 @@
         <v>7</v>
       </c>
       <c r="B109" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="C109" t="s">
-        <v>155</v>
-      </c>
-      <c r="D109" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="E109" s="6"/>
+        <v>139</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="E109" s="4"/>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110">
@@ -2611,15 +2494,15 @@
         <v>8</v>
       </c>
       <c r="B110" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="C110" t="s">
-        <v>157</v>
-      </c>
-      <c r="D110" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="E110" s="6"/>
+        <v>141</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E110" s="4"/>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111">
@@ -2627,15 +2510,15 @@
         <v>9</v>
       </c>
       <c r="B111" t="s">
-        <v>264</v>
+        <v>232</v>
       </c>
       <c r="C111" t="s">
-        <v>151</v>
-      </c>
-      <c r="D111" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="E111" s="6"/>
+        <v>135</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="E111" s="4"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112">
@@ -2643,15 +2526,15 @@
         <v>10</v>
       </c>
       <c r="B112" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="C112" t="s">
-        <v>159</v>
-      </c>
-      <c r="D112" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="E112" s="6"/>
+        <v>143</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E112" s="4"/>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113">
@@ -2659,15 +2542,15 @@
         <v>11</v>
       </c>
       <c r="B113" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="C113" t="s">
-        <v>161</v>
-      </c>
-      <c r="D113" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="E113" s="6"/>
+        <v>145</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="E113" s="4"/>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114">
@@ -2675,29 +2558,29 @@
         <v>12</v>
       </c>
       <c r="B114" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="C114" t="s">
-        <v>163</v>
-      </c>
-      <c r="D114" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="E114" s="6"/>
+        <v>147</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="E114" s="4"/>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A115" s="1">
+      <c r="A115" s="11">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="B115" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D115" s="4" t="s">
-        <v>262</v>
+      <c r="B115" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="C115" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="D115" s="12" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
@@ -2706,15 +2589,15 @@
         <v>14</v>
       </c>
       <c r="B116" t="s">
-        <v>166</v>
+        <v>148</v>
       </c>
       <c r="C116" t="s">
-        <v>167</v>
-      </c>
-      <c r="D116" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="E116" s="6"/>
+        <v>149</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E116" s="4"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117">
@@ -2722,15 +2605,15 @@
         <v>15</v>
       </c>
       <c r="B117" t="s">
-        <v>168</v>
+        <v>150</v>
       </c>
       <c r="C117" t="s">
-        <v>169</v>
-      </c>
-      <c r="D117" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="E117" s="6"/>
+        <v>151</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="E117" s="4"/>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118">
@@ -2738,50 +2621,24 @@
         <v>16</v>
       </c>
       <c r="B118" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="C118" t="s">
-        <v>171</v>
-      </c>
-      <c r="D118" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="E118" s="6"/>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A119" s="1">
-        <v>17</v>
-      </c>
-      <c r="B119" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="D119" s="4" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A121" s="8" t="s">
-        <v>261</v>
-      </c>
-      <c r="B121" s="8"/>
-      <c r="C121" s="8"/>
-      <c r="D121" s="8"/>
+        <v>153</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E118" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A72:D72"/>
+  <mergeCells count="6">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A52:D52"/>
     <mergeCell ref="A98:D98"/>
     <mergeCell ref="A78:D78"/>
     <mergeCell ref="A100:D100"/>
-    <mergeCell ref="A121:D121"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A50:D50"/>
-    <mergeCell ref="A52:D52"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="55" orientation="landscape" r:id="rId1"/>

</xml_diff>